<commit_message>
chore: update midweek data workbook
</commit_message>
<xml_diff>
--- a/Midweek_Data.xlsx
+++ b/Midweek_Data.xlsx
@@ -484,13 +484,13 @@
         <v>5</v>
       </c>
       <c r="D3" t="n">
-        <v>31</v>
+        <v>15</v>
       </c>
       <c r="E3" t="n">
-        <v>1289</v>
+        <v>2040</v>
       </c>
       <c r="F3" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="4">
@@ -508,13 +508,13 @@
         <v>33</v>
       </c>
       <c r="D4" t="n">
-        <v>74</v>
+        <v>88</v>
       </c>
       <c r="E4" t="n">
-        <v>5241</v>
+        <v>2829</v>
       </c>
       <c r="F4" t="n">
-        <v>25</v>
+        <v>27</v>
       </c>
     </row>
     <row r="5">
@@ -532,10 +532,10 @@
         <v>13</v>
       </c>
       <c r="D5" t="n">
-        <v>31</v>
+        <v>39</v>
       </c>
       <c r="E5" t="n">
-        <v>1106</v>
+        <v>2383</v>
       </c>
       <c r="F5" t="n">
         <v>5</v>
@@ -556,13 +556,13 @@
         <v>15</v>
       </c>
       <c r="D6" t="n">
-        <v>19</v>
+        <v>30</v>
       </c>
       <c r="E6" t="n">
-        <v>3478</v>
+        <v>2455</v>
       </c>
       <c r="F6" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
     </row>
     <row r="7">
@@ -580,13 +580,13 @@
         <v>28</v>
       </c>
       <c r="D7" t="n">
-        <v>116</v>
+        <v>119</v>
       </c>
       <c r="E7" t="n">
-        <v>1761</v>
+        <v>3154</v>
       </c>
       <c r="F7" t="n">
-        <v>18</v>
+        <v>20</v>
       </c>
     </row>
     <row r="8">
@@ -604,13 +604,13 @@
         <v>5</v>
       </c>
       <c r="D8" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="E8" t="n">
-        <v>0</v>
+        <v>205</v>
       </c>
       <c r="F8" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="9">
@@ -625,16 +625,16 @@
         </is>
       </c>
       <c r="C9" t="n">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="D9" t="n">
-        <v>162</v>
+        <v>165</v>
       </c>
       <c r="E9" t="n">
-        <v>2562</v>
+        <v>2279</v>
       </c>
       <c r="F9" t="n">
-        <v>36</v>
+        <v>37</v>
       </c>
     </row>
     <row r="10">
@@ -652,13 +652,13 @@
         <v>42</v>
       </c>
       <c r="D10" t="n">
-        <v>109</v>
+        <v>64</v>
       </c>
       <c r="E10" t="n">
-        <v>1314</v>
+        <v>471</v>
       </c>
       <c r="F10" t="n">
-        <v>28</v>
+        <v>19</v>
       </c>
     </row>
     <row r="11">
@@ -676,13 +676,13 @@
         <v>19</v>
       </c>
       <c r="D11" t="n">
-        <v>93</v>
+        <v>63</v>
       </c>
       <c r="E11" t="n">
-        <v>1062</v>
+        <v>1081</v>
       </c>
       <c r="F11" t="n">
-        <v>13</v>
+        <v>11</v>
       </c>
     </row>
     <row r="12">
@@ -700,13 +700,13 @@
         <v>50</v>
       </c>
       <c r="D12" t="n">
-        <v>99</v>
+        <v>77</v>
       </c>
       <c r="E12" t="n">
-        <v>3081</v>
+        <v>3398</v>
       </c>
       <c r="F12" t="n">
-        <v>21</v>
+        <v>20</v>
       </c>
     </row>
     <row r="13">
@@ -721,16 +721,16 @@
         </is>
       </c>
       <c r="C13" t="n">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="D13" t="n">
-        <v>127</v>
+        <v>138</v>
       </c>
       <c r="E13" t="n">
-        <v>2974</v>
+        <v>3645</v>
       </c>
       <c r="F13" t="n">
-        <v>33</v>
+        <v>39</v>
       </c>
     </row>
     <row r="14">
@@ -748,13 +748,13 @@
         <v>42</v>
       </c>
       <c r="D14" t="n">
-        <v>116</v>
+        <v>100</v>
       </c>
       <c r="E14" t="n">
-        <v>913</v>
+        <v>596</v>
       </c>
       <c r="F14" t="n">
-        <v>27</v>
+        <v>26</v>
       </c>
     </row>
     <row r="15">
@@ -772,13 +772,13 @@
         <v>31</v>
       </c>
       <c r="D15" t="n">
-        <v>86</v>
+        <v>118</v>
       </c>
       <c r="E15" t="n">
-        <v>1731</v>
+        <v>1813</v>
       </c>
       <c r="F15" t="n">
-        <v>21</v>
+        <v>22</v>
       </c>
     </row>
     <row r="16">
@@ -796,13 +796,13 @@
         <v>30</v>
       </c>
       <c r="D16" t="n">
-        <v>77</v>
+        <v>68</v>
       </c>
       <c r="E16" t="n">
-        <v>2277</v>
+        <v>2259</v>
       </c>
       <c r="F16" t="n">
-        <v>18</v>
+        <v>15</v>
       </c>
     </row>
   </sheetData>
@@ -888,21 +888,21 @@
         <v>6</v>
       </c>
       <c r="D3" t="n">
-        <v>43</v>
+        <v>26</v>
       </c>
       <c r="E3" t="n">
-        <v>393</v>
+        <v>570</v>
       </c>
       <c r="F3" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>6/6</t>
+          <t>5/6</t>
         </is>
       </c>
       <c r="H3" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I3" t="inlineStr"/>
     </row>
@@ -954,21 +954,21 @@
         <v>4</v>
       </c>
       <c r="D5" t="n">
-        <v>31</v>
+        <v>22</v>
       </c>
       <c r="E5" t="n">
-        <v>165</v>
+        <v>175</v>
       </c>
       <c r="F5" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>4/4</t>
+          <t>3/4</t>
         </is>
       </c>
       <c r="H5" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I5" t="inlineStr"/>
     </row>
@@ -987,10 +987,10 @@
         <v>5</v>
       </c>
       <c r="D6" t="n">
-        <v>19</v>
+        <v>15</v>
       </c>
       <c r="E6" t="n">
-        <v>504</v>
+        <v>336</v>
       </c>
       <c r="F6" t="n">
         <v>3</v>
@@ -1152,10 +1152,10 @@
         <v>4</v>
       </c>
       <c r="D4" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="E4" t="n">
-        <v>25</v>
+        <v>46</v>
       </c>
       <c r="F4" t="n">
         <v>2</v>
@@ -1185,21 +1185,21 @@
         <v>7</v>
       </c>
       <c r="D5" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="E5" t="n">
-        <v>0</v>
+        <v>70</v>
       </c>
       <c r="F5" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>0/7</t>
+          <t>2/7</t>
         </is>
       </c>
       <c r="H5" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="I5" t="inlineStr"/>
     </row>
@@ -1218,10 +1218,10 @@
         <v>2</v>
       </c>
       <c r="D6" t="n">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="E6" t="n">
-        <v>110</v>
+        <v>40</v>
       </c>
       <c r="F6" t="n">
         <v>2</v>
@@ -1251,10 +1251,10 @@
         <v>2</v>
       </c>
       <c r="D7" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="E7" t="n">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="F7" t="n">
         <v>1</v>
@@ -1284,21 +1284,21 @@
         <v>3</v>
       </c>
       <c r="D8" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="E8" t="n">
-        <v>1050</v>
+        <v>0</v>
       </c>
       <c r="F8" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>1/3</t>
+          <t>0/3</t>
         </is>
       </c>
       <c r="H8" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="I8" t="inlineStr"/>
     </row>
@@ -1317,10 +1317,10 @@
         <v>5</v>
       </c>
       <c r="D9" t="n">
-        <v>14</v>
+        <v>6</v>
       </c>
       <c r="E9" t="n">
-        <v>100</v>
+        <v>1870</v>
       </c>
       <c r="F9" t="n">
         <v>2</v>
@@ -1350,10 +1350,10 @@
         <v>2</v>
       </c>
       <c r="D10" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="E10" t="n">
-        <v>700</v>
+        <v>400</v>
       </c>
       <c r="F10" t="n">
         <v>1</v>
@@ -1383,21 +1383,21 @@
         <v>4</v>
       </c>
       <c r="D11" t="n">
-        <v>12</v>
+        <v>5</v>
       </c>
       <c r="E11" t="n">
-        <v>55</v>
+        <v>15</v>
       </c>
       <c r="F11" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>2/4</t>
+          <t>1/4</t>
         </is>
       </c>
       <c r="H11" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="I11" t="inlineStr"/>
     </row>
@@ -1416,21 +1416,21 @@
         <v>2</v>
       </c>
       <c r="D12" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="E12" t="n">
-        <v>50</v>
+        <v>40</v>
       </c>
       <c r="F12" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>2/2</t>
+          <t>1/2</t>
         </is>
       </c>
       <c r="H12" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I12" t="inlineStr"/>
     </row>
@@ -1452,7 +1452,7 @@
         <v>7</v>
       </c>
       <c r="E13" t="n">
-        <v>270</v>
+        <v>100</v>
       </c>
       <c r="F13" t="n">
         <v>3</v>
@@ -1485,7 +1485,7 @@
         <v>23</v>
       </c>
       <c r="E14" t="n">
-        <v>706</v>
+        <v>807</v>
       </c>
       <c r="F14" t="n">
         <v>5</v>
@@ -1614,21 +1614,21 @@
         <v>3</v>
       </c>
       <c r="D3" t="n">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="E3" t="n">
-        <v>70</v>
+        <v>35</v>
       </c>
       <c r="F3" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>3/3</t>
+          <t>2/3</t>
         </is>
       </c>
       <c r="H3" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I3" t="inlineStr"/>
     </row>
@@ -1647,10 +1647,10 @@
         <v>3</v>
       </c>
       <c r="D4" t="n">
-        <v>12</v>
+        <v>16</v>
       </c>
       <c r="E4" t="n">
-        <v>100</v>
+        <v>180</v>
       </c>
       <c r="F4" t="n">
         <v>3</v>
@@ -1677,20 +1677,20 @@
         </is>
       </c>
       <c r="C5" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="D5" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="E5" t="n">
-        <v>1940</v>
+        <v>125</v>
       </c>
       <c r="F5" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>4/4</t>
+          <t>6/6</t>
         </is>
       </c>
       <c r="H5" t="n">
@@ -1713,10 +1713,10 @@
         <v>1</v>
       </c>
       <c r="D6" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="E6" t="n">
-        <v>50</v>
+        <v>150</v>
       </c>
       <c r="F6" t="n">
         <v>1</v>
@@ -1746,7 +1746,7 @@
         <v>1</v>
       </c>
       <c r="D7" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="E7" t="n">
         <v>50</v>
@@ -1782,7 +1782,7 @@
         <v>17</v>
       </c>
       <c r="E8" t="n">
-        <v>165</v>
+        <v>115</v>
       </c>
       <c r="F8" t="n">
         <v>3</v>
@@ -1812,10 +1812,10 @@
         <v>2</v>
       </c>
       <c r="D9" t="n">
-        <v>10</v>
+        <v>7</v>
       </c>
       <c r="E9" t="n">
-        <v>70</v>
+        <v>75</v>
       </c>
       <c r="F9" t="n">
         <v>2</v>
@@ -1845,10 +1845,10 @@
         <v>2</v>
       </c>
       <c r="D10" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="E10" t="n">
-        <v>35</v>
+        <v>40</v>
       </c>
       <c r="F10" t="n">
         <v>2</v>
@@ -1881,7 +1881,7 @@
         <v>11</v>
       </c>
       <c r="E11" t="n">
-        <v>138</v>
+        <v>60</v>
       </c>
       <c r="F11" t="n">
         <v>4</v>
@@ -1911,21 +1911,21 @@
         <v>2</v>
       </c>
       <c r="D12" t="n">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="E12" t="n">
-        <v>15</v>
+        <v>55</v>
       </c>
       <c r="F12" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>1/2</t>
+          <t>2/2</t>
         </is>
       </c>
       <c r="H12" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I12" t="inlineStr"/>
     </row>
@@ -1944,21 +1944,21 @@
         <v>5</v>
       </c>
       <c r="D13" t="n">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="E13" t="n">
-        <v>210</v>
+        <v>230</v>
       </c>
       <c r="F13" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>5/5</t>
+          <t>4/5</t>
         </is>
       </c>
       <c r="H13" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I13" t="inlineStr"/>
     </row>
@@ -1977,21 +1977,21 @@
         <v>2</v>
       </c>
       <c r="D14" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="E14" t="n">
-        <v>0</v>
+        <v>20</v>
       </c>
       <c r="F14" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>0/2</t>
+          <t>1/2</t>
         </is>
       </c>
       <c r="H14" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="I14" t="inlineStr"/>
     </row>
@@ -2010,21 +2010,21 @@
         <v>3</v>
       </c>
       <c r="D15" t="n">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="E15" t="n">
-        <v>36</v>
+        <v>2355</v>
       </c>
       <c r="F15" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>1/3</t>
+          <t>3/3</t>
         </is>
       </c>
       <c r="H15" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="I15" t="inlineStr"/>
     </row>
@@ -2043,21 +2043,21 @@
         <v>2</v>
       </c>
       <c r="D16" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="E16" t="n">
-        <v>0</v>
+        <v>50</v>
       </c>
       <c r="F16" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>0/2</t>
+          <t>2/2</t>
         </is>
       </c>
       <c r="H16" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="I16" t="inlineStr"/>
     </row>
@@ -2109,10 +2109,10 @@
         <v>3</v>
       </c>
       <c r="D18" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="E18" t="n">
-        <v>95</v>
+        <v>105</v>
       </c>
       <c r="F18" t="n">
         <v>3</v>
@@ -2241,21 +2241,21 @@
         <v>3</v>
       </c>
       <c r="D3" t="n">
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="E3" t="n">
-        <v>0</v>
+        <v>50</v>
       </c>
       <c r="F3" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>0/3</t>
+          <t>2/3</t>
         </is>
       </c>
       <c r="H3" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="I3" t="inlineStr"/>
     </row>
@@ -2274,7 +2274,7 @@
         <v>3</v>
       </c>
       <c r="D4" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="E4" t="n">
         <v>45</v>
@@ -2307,21 +2307,21 @@
         <v>2</v>
       </c>
       <c r="D5" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="E5" t="n">
-        <v>25</v>
+        <v>20</v>
       </c>
       <c r="F5" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>2/2</t>
+          <t>1/2</t>
         </is>
       </c>
       <c r="H5" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I5" t="inlineStr"/>
     </row>
@@ -2340,21 +2340,21 @@
         <v>2</v>
       </c>
       <c r="D6" t="n">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="E6" t="n">
-        <v>40</v>
+        <v>75</v>
       </c>
       <c r="F6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>1/2</t>
+          <t>2/2</t>
         </is>
       </c>
       <c r="H6" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I6" t="inlineStr"/>
     </row>
@@ -2373,10 +2373,10 @@
         <v>2</v>
       </c>
       <c r="D7" t="n">
-        <v>9</v>
+        <v>5</v>
       </c>
       <c r="E7" t="n">
-        <v>35</v>
+        <v>25</v>
       </c>
       <c r="F7" t="n">
         <v>2</v>
@@ -2406,10 +2406,10 @@
         <v>2</v>
       </c>
       <c r="D8" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="E8" t="n">
-        <v>30</v>
+        <v>5</v>
       </c>
       <c r="F8" t="n">
         <v>1</v>
@@ -2439,21 +2439,21 @@
         <v>1</v>
       </c>
       <c r="D9" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="E9" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="F9" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>1/1</t>
+          <t>0/1</t>
         </is>
       </c>
       <c r="H9" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I9" t="inlineStr"/>
     </row>
@@ -2472,21 +2472,21 @@
         <v>3</v>
       </c>
       <c r="D10" t="n">
-        <v>4</v>
+        <v>11</v>
       </c>
       <c r="E10" t="n">
-        <v>20</v>
+        <v>50</v>
       </c>
       <c r="F10" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>1/3</t>
+          <t>3/3</t>
         </is>
       </c>
       <c r="H10" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="I10" t="inlineStr"/>
     </row>
@@ -2505,10 +2505,10 @@
         <v>3</v>
       </c>
       <c r="D11" t="n">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="E11" t="n">
-        <v>90</v>
+        <v>100</v>
       </c>
       <c r="F11" t="n">
         <v>2</v>
@@ -2571,21 +2571,21 @@
         <v>3</v>
       </c>
       <c r="D13" t="n">
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="E13" t="n">
-        <v>30</v>
+        <v>0</v>
       </c>
       <c r="F13" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>1/3</t>
+          <t>0/3</t>
         </is>
       </c>
       <c r="H13" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="I13" t="inlineStr"/>
     </row>
@@ -2604,10 +2604,10 @@
         <v>3</v>
       </c>
       <c r="D14" t="n">
-        <v>13</v>
+        <v>8</v>
       </c>
       <c r="E14" t="n">
-        <v>55</v>
+        <v>50</v>
       </c>
       <c r="F14" t="n">
         <v>3</v>
@@ -2637,21 +2637,21 @@
         <v>7</v>
       </c>
       <c r="D15" t="n">
-        <v>28</v>
+        <v>24</v>
       </c>
       <c r="E15" t="n">
-        <v>160</v>
+        <v>126</v>
       </c>
       <c r="F15" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>7/7</t>
+          <t>6/7</t>
         </is>
       </c>
       <c r="H15" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I15" t="inlineStr"/>
     </row>
@@ -2670,21 +2670,21 @@
         <v>2</v>
       </c>
       <c r="D16" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="E16" t="n">
-        <v>215</v>
+        <v>0</v>
       </c>
       <c r="F16" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>1/2</t>
+          <t>0/2</t>
         </is>
       </c>
       <c r="H16" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I16" t="inlineStr"/>
     </row>
@@ -2703,10 +2703,10 @@
         <v>2</v>
       </c>
       <c r="D17" t="n">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="E17" t="n">
-        <v>140</v>
+        <v>50</v>
       </c>
       <c r="F17" t="n">
         <v>2</v>
@@ -2736,21 +2736,21 @@
         <v>2</v>
       </c>
       <c r="D18" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="E18" t="n">
-        <v>22</v>
+        <v>0</v>
       </c>
       <c r="F18" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>1/2</t>
+          <t>0/2</t>
         </is>
       </c>
       <c r="H18" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I18" t="inlineStr"/>
     </row>
@@ -2796,7 +2796,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I12"/>
+  <dimension ref="A1:I13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2868,10 +2868,10 @@
         <v>4</v>
       </c>
       <c r="D3" t="n">
-        <v>12</v>
+        <v>7</v>
       </c>
       <c r="E3" t="n">
-        <v>259</v>
+        <v>345</v>
       </c>
       <c r="F3" t="n">
         <v>1</v>
@@ -2904,7 +2904,7 @@
         <v>4</v>
       </c>
       <c r="E4" t="n">
-        <v>20</v>
+        <v>30</v>
       </c>
       <c r="F4" t="n">
         <v>1</v>
@@ -2934,21 +2934,21 @@
         <v>4</v>
       </c>
       <c r="D5" t="n">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="E5" t="n">
-        <v>245</v>
+        <v>140</v>
       </c>
       <c r="F5" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>4/4</t>
+          <t>3/4</t>
         </is>
       </c>
       <c r="H5" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I5" t="inlineStr"/>
     </row>
@@ -2970,7 +2970,7 @@
         <v>8</v>
       </c>
       <c r="E6" t="n">
-        <v>342</v>
+        <v>110</v>
       </c>
       <c r="F6" t="n">
         <v>3</v>
@@ -3000,10 +3000,10 @@
         <v>2</v>
       </c>
       <c r="D7" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E7" t="n">
-        <v>160</v>
+        <v>180</v>
       </c>
       <c r="F7" t="n">
         <v>1</v>
@@ -3036,18 +3036,18 @@
         <v>5</v>
       </c>
       <c r="E8" t="n">
-        <v>50</v>
+        <v>40</v>
       </c>
       <c r="F8" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>1/3</t>
+          <t>2/3</t>
         </is>
       </c>
       <c r="H8" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="I8" t="inlineStr"/>
     </row>
@@ -3066,10 +3066,10 @@
         <v>7</v>
       </c>
       <c r="D9" t="n">
-        <v>22</v>
+        <v>28</v>
       </c>
       <c r="E9" t="n">
-        <v>435</v>
+        <v>283</v>
       </c>
       <c r="F9" t="n">
         <v>7</v>
@@ -3099,10 +3099,10 @@
         <v>6</v>
       </c>
       <c r="D10" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E10" t="n">
-        <v>160</v>
+        <v>230</v>
       </c>
       <c r="F10" t="n">
         <v>2</v>
@@ -3135,7 +3135,7 @@
         <v>7</v>
       </c>
       <c r="E11" t="n">
-        <v>60</v>
+        <v>70</v>
       </c>
       <c r="F11" t="n">
         <v>1</v>
@@ -3153,31 +3153,55 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
+          <t>Council Service</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr"/>
+      <c r="D12" t="n">
+        <v>33</v>
+      </c>
+      <c r="E12" t="n">
+        <v>385</v>
+      </c>
+      <c r="F12" t="n">
+        <v>1</v>
+      </c>
+      <c r="G12" t="inlineStr"/>
+      <c r="H12" t="inlineStr"/>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>Council Service</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="C12">
-        <f>SUM(C3:C11)</f>
-        <v/>
-      </c>
-      <c r="D12">
-        <f>SUM(D3:D11)</f>
-        <v/>
-      </c>
-      <c r="E12">
-        <f>SUM(E3:E11)</f>
-        <v/>
-      </c>
-      <c r="F12">
-        <f>SUM(F3:F11)</f>
-        <v/>
-      </c>
-      <c r="G12">
-        <f>F12&amp;"/"&amp;C12</f>
-        <v/>
-      </c>
-      <c r="H12">
-        <f>SUM(H3:H11)</f>
+      <c r="C13">
+        <f>SUM(C3:C12)</f>
+        <v/>
+      </c>
+      <c r="D13">
+        <f>SUM(D3:D12)</f>
+        <v/>
+      </c>
+      <c r="E13">
+        <f>SUM(E3:E12)</f>
+        <v/>
+      </c>
+      <c r="F13">
+        <f>SUM(F3:F12)</f>
+        <v/>
+      </c>
+      <c r="G13">
+        <f>F13&amp;"/"&amp;C13</f>
+        <v/>
+      </c>
+      <c r="H13">
+        <f>SUM(H3:H12)</f>
         <v/>
       </c>
     </row>
@@ -3264,21 +3288,21 @@
         <v>5</v>
       </c>
       <c r="D3" t="n">
-        <v>16</v>
+        <v>6</v>
       </c>
       <c r="E3" t="n">
-        <v>80</v>
+        <v>60</v>
       </c>
       <c r="F3" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>4/5</t>
+          <t>2/5</t>
         </is>
       </c>
       <c r="H3" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="I3" t="inlineStr"/>
     </row>
@@ -3294,24 +3318,24 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="D4" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="E4" t="n">
-        <v>0</v>
+        <v>19</v>
       </c>
       <c r="F4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>0/0</t>
+          <t>1/2</t>
         </is>
       </c>
       <c r="H4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I4" t="inlineStr"/>
     </row>
@@ -3327,24 +3351,24 @@
         </is>
       </c>
       <c r="C5" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D5" t="n">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="E5" t="n">
-        <v>50</v>
+        <v>215</v>
       </c>
       <c r="F5" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>1/4</t>
+          <t>2/3</t>
         </is>
       </c>
       <c r="H5" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="I5" t="inlineStr"/>
     </row>
@@ -3360,24 +3384,24 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D6" t="n">
-        <v>19</v>
+        <v>7</v>
       </c>
       <c r="E6" t="n">
-        <v>1717</v>
+        <v>440</v>
       </c>
       <c r="F6" t="n">
         <v>2</v>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>2/2</t>
+          <t>2/3</t>
         </is>
       </c>
       <c r="H6" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I6" t="inlineStr"/>
     </row>
@@ -3393,20 +3417,20 @@
         </is>
       </c>
       <c r="C7" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D7" t="n">
-        <v>9</v>
+        <v>3</v>
       </c>
       <c r="E7" t="n">
-        <v>80</v>
+        <v>30</v>
       </c>
       <c r="F7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>2/3</t>
+          <t>1/2</t>
         </is>
       </c>
       <c r="H7" t="n">
@@ -3426,24 +3450,24 @@
         </is>
       </c>
       <c r="C8" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D8" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="E8" t="n">
-        <v>140</v>
+        <v>105</v>
       </c>
       <c r="F8" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>2/2</t>
+          <t>1/3</t>
         </is>
       </c>
       <c r="H8" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="I8" t="inlineStr"/>
     </row>
@@ -3459,24 +3483,24 @@
         </is>
       </c>
       <c r="C9" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="D9" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E9" t="n">
-        <v>60</v>
+        <v>100</v>
       </c>
       <c r="F9" t="n">
         <v>1</v>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>1/4</t>
+          <t>1/2</t>
         </is>
       </c>
       <c r="H9" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="I9" t="inlineStr"/>
     </row>
@@ -3492,24 +3516,24 @@
         </is>
       </c>
       <c r="C10" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D10" t="n">
-        <v>13</v>
+        <v>8</v>
       </c>
       <c r="E10" t="n">
-        <v>85</v>
+        <v>50</v>
       </c>
       <c r="F10" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>4/4</t>
+          <t>2/3</t>
         </is>
       </c>
       <c r="H10" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I10" t="inlineStr"/>
     </row>
@@ -3525,24 +3549,24 @@
         </is>
       </c>
       <c r="C11" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D11" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E11" t="n">
-        <v>35</v>
+        <v>30</v>
       </c>
       <c r="F11" t="n">
         <v>1</v>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>1/2</t>
+          <t>1/3</t>
         </is>
       </c>
       <c r="H11" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I11" t="inlineStr"/>
     </row>
@@ -3558,24 +3582,24 @@
         </is>
       </c>
       <c r="C12" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="D12" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="E12" t="n">
-        <v>0</v>
+        <v>50</v>
       </c>
       <c r="F12" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>0/0</t>
+          <t>1/3</t>
         </is>
       </c>
       <c r="H12" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="I12" t="inlineStr"/>
     </row>
@@ -3591,24 +3615,24 @@
         </is>
       </c>
       <c r="C13" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="D13" t="n">
-        <v>3</v>
+        <v>17</v>
       </c>
       <c r="E13" t="n">
-        <v>30</v>
+        <v>1160</v>
       </c>
       <c r="F13" t="n">
         <v>1</v>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>1/4</t>
+          <t>1/1</t>
         </is>
       </c>
       <c r="H13" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="I13" t="inlineStr"/>
     </row>
@@ -3726,21 +3750,21 @@
         <v>3</v>
       </c>
       <c r="D3" t="n">
-        <v>20</v>
+        <v>9</v>
       </c>
       <c r="E3" t="n">
-        <v>1127</v>
+        <v>1660</v>
       </c>
       <c r="F3" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>3/3</t>
+          <t>2/3</t>
         </is>
       </c>
       <c r="H3" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I3" t="inlineStr"/>
     </row>
@@ -3759,10 +3783,10 @@
         <v>1</v>
       </c>
       <c r="D4" t="n">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="E4" t="n">
-        <v>92</v>
+        <v>80</v>
       </c>
       <c r="F4" t="n">
         <v>1</v>
@@ -3792,10 +3816,10 @@
         <v>1</v>
       </c>
       <c r="D5" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E5" t="n">
-        <v>70</v>
+        <v>300</v>
       </c>
       <c r="F5" t="n">
         <v>1</v>
@@ -3924,10 +3948,10 @@
         <v>1</v>
       </c>
       <c r="D3" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="E3" t="n">
-        <v>20</v>
+        <v>10</v>
       </c>
       <c r="F3" t="n">
         <v>1</v>
@@ -3957,10 +3981,10 @@
         <v>6</v>
       </c>
       <c r="D4" t="n">
-        <v>14</v>
+        <v>19</v>
       </c>
       <c r="E4" t="n">
-        <v>85</v>
+        <v>50</v>
       </c>
       <c r="F4" t="n">
         <v>6</v>
@@ -3990,10 +4014,10 @@
         <v>1</v>
       </c>
       <c r="D5" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E5" t="n">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="F5" t="n">
         <v>1</v>
@@ -4023,21 +4047,21 @@
         <v>3</v>
       </c>
       <c r="D6" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="E6" t="n">
-        <v>85</v>
+        <v>50</v>
       </c>
       <c r="F6" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>3/3</t>
+          <t>2/3</t>
         </is>
       </c>
       <c r="H6" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I6" t="inlineStr"/>
     </row>
@@ -4056,10 +4080,10 @@
         <v>5</v>
       </c>
       <c r="D7" t="n">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="E7" t="n">
-        <v>78</v>
+        <v>69</v>
       </c>
       <c r="F7" t="n">
         <v>5</v>
@@ -4122,10 +4146,10 @@
         <v>6</v>
       </c>
       <c r="D9" t="n">
-        <v>18</v>
+        <v>24</v>
       </c>
       <c r="E9" t="n">
-        <v>4903</v>
+        <v>2216</v>
       </c>
       <c r="F9" t="n">
         <v>6</v>
@@ -4155,21 +4179,21 @@
         <v>4</v>
       </c>
       <c r="D10" t="n">
-        <v>5</v>
+        <v>11</v>
       </c>
       <c r="E10" t="n">
-        <v>30</v>
+        <v>379</v>
       </c>
       <c r="F10" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>2/4</t>
+          <t>4/4</t>
         </is>
       </c>
       <c r="H10" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="I10" t="inlineStr"/>
     </row>
@@ -4221,21 +4245,21 @@
         <v>2</v>
       </c>
       <c r="D12" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="E12" t="n">
-        <v>0</v>
+        <v>20</v>
       </c>
       <c r="F12" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>0/2</t>
+          <t>1/2</t>
         </is>
       </c>
       <c r="H12" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="I12" t="inlineStr"/>
     </row>
@@ -4353,10 +4377,10 @@
         <v>3</v>
       </c>
       <c r="D3" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="E3" t="n">
-        <v>158</v>
+        <v>148</v>
       </c>
       <c r="F3" t="n">
         <v>1</v>
@@ -4386,21 +4410,21 @@
         <v>2</v>
       </c>
       <c r="D4" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="E4" t="n">
-        <v>0</v>
+        <v>2000</v>
       </c>
       <c r="F4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>0/2</t>
+          <t>1/2</t>
         </is>
       </c>
       <c r="H4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="I4" t="inlineStr"/>
     </row>
@@ -4452,21 +4476,21 @@
         <v>1</v>
       </c>
       <c r="D6" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="E6" t="n">
-        <v>20</v>
+        <v>0</v>
       </c>
       <c r="F6" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>1/1</t>
+          <t>0/1</t>
         </is>
       </c>
       <c r="H6" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I6" t="inlineStr"/>
     </row>
@@ -4485,10 +4509,10 @@
         <v>1</v>
       </c>
       <c r="D7" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="E7" t="n">
-        <v>810</v>
+        <v>112</v>
       </c>
       <c r="F7" t="n">
         <v>1</v>
@@ -4518,10 +4542,10 @@
         <v>5</v>
       </c>
       <c r="D8" t="n">
-        <v>15</v>
+        <v>22</v>
       </c>
       <c r="E8" t="n">
-        <v>118</v>
+        <v>123</v>
       </c>
       <c r="F8" t="n">
         <v>2</v>
@@ -4650,10 +4674,10 @@
         <v>5</v>
       </c>
       <c r="D3" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="E3" t="n">
-        <v>3204</v>
+        <v>2227</v>
       </c>
       <c r="F3" t="n">
         <v>2</v>
@@ -4683,21 +4707,21 @@
         <v>6</v>
       </c>
       <c r="D4" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="E4" t="n">
-        <v>170</v>
+        <v>112</v>
       </c>
       <c r="F4" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>3/6</t>
+          <t>1/6</t>
         </is>
       </c>
       <c r="H4" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="I4" t="inlineStr"/>
     </row>
@@ -4716,10 +4740,10 @@
         <v>4</v>
       </c>
       <c r="D5" t="n">
-        <v>3</v>
+        <v>11</v>
       </c>
       <c r="E5" t="n">
-        <v>104</v>
+        <v>116</v>
       </c>
       <c r="F5" t="n">
         <v>1</v>
@@ -4845,10 +4869,10 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D3" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="E3" t="n">
         <v>20</v>
@@ -4858,11 +4882,11 @@
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>1/4</t>
+          <t>1/3</t>
         </is>
       </c>
       <c r="H3" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="I3" t="inlineStr"/>
     </row>
@@ -4878,20 +4902,20 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D4" t="n">
-        <v>16</v>
+        <v>23</v>
       </c>
       <c r="E4" t="n">
-        <v>409</v>
+        <v>480</v>
       </c>
       <c r="F4" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>3/3</t>
+          <t>4/4</t>
         </is>
       </c>
       <c r="H4" t="n">
@@ -4914,21 +4938,21 @@
         <v>6</v>
       </c>
       <c r="D5" t="n">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="E5" t="n">
-        <v>201</v>
+        <v>750</v>
       </c>
       <c r="F5" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>2/6</t>
+          <t>3/6</t>
         </is>
       </c>
       <c r="H5" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="I5" t="inlineStr"/>
     </row>
@@ -4947,10 +4971,10 @@
         <v>4</v>
       </c>
       <c r="D6" t="n">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="E6" t="n">
-        <v>45</v>
+        <v>250</v>
       </c>
       <c r="F6" t="n">
         <v>3</v>
@@ -4980,10 +5004,10 @@
         <v>4</v>
       </c>
       <c r="D7" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="E7" t="n">
-        <v>120</v>
+        <v>650</v>
       </c>
       <c r="F7" t="n">
         <v>2</v>
@@ -5013,10 +5037,10 @@
         <v>4</v>
       </c>
       <c r="D8" t="n">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="E8" t="n">
-        <v>172</v>
+        <v>168</v>
       </c>
       <c r="F8" t="n">
         <v>3</v>
@@ -5046,10 +5070,10 @@
         <v>3</v>
       </c>
       <c r="D9" t="n">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="E9" t="n">
-        <v>160</v>
+        <v>305</v>
       </c>
       <c r="F9" t="n">
         <v>3</v>
@@ -5072,10 +5096,10 @@
       </c>
       <c r="B10" t="inlineStr"/>
       <c r="D10" t="n">
-        <v>36</v>
+        <v>31</v>
       </c>
       <c r="E10" t="n">
-        <v>634</v>
+        <v>531</v>
       </c>
       <c r="F10" t="n">
         <v>1</v>
@@ -5235,21 +5259,21 @@
         <v>2</v>
       </c>
       <c r="D4" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="E4" t="n">
-        <v>0</v>
+        <v>205</v>
       </c>
       <c r="F4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>0/2</t>
+          <t>1/2</t>
         </is>
       </c>
       <c r="H4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="I4" t="inlineStr"/>
     </row>
@@ -5328,7 +5352,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I13"/>
+  <dimension ref="A1:I12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -5400,10 +5424,10 @@
         <v>2</v>
       </c>
       <c r="D3" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E3" t="n">
-        <v>80</v>
+        <v>60</v>
       </c>
       <c r="F3" t="n">
         <v>2</v>
@@ -5421,62 +5445,62 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Adabraka</t>
+          <t>Arena</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Emmanuel Otiboe</t>
+          <t>Zephaniah Lartey</t>
         </is>
       </c>
       <c r="C4" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="D4" t="n">
-        <v>28</v>
+        <v>22</v>
       </c>
       <c r="E4" t="n">
-        <v>272</v>
+        <v>230</v>
       </c>
       <c r="F4" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>4/5</t>
+          <t>6/6</t>
         </is>
       </c>
       <c r="H4" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Arena</t>
+          <t>ATU Church</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Zephaniah Lartey</t>
+          <t>James Pekyie</t>
         </is>
       </c>
       <c r="C5" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="D5" t="n">
-        <v>26</v>
+        <v>23</v>
       </c>
       <c r="E5" t="n">
-        <v>225</v>
+        <v>182</v>
       </c>
       <c r="F5" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>6/6</t>
+          <t>5/5</t>
         </is>
       </c>
       <c r="H5" t="n">
@@ -5487,29 +5511,29 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>ATU Church</t>
+          <t>ATU Main Campus</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>James Pekyie</t>
+          <t>Racheal Boamah</t>
         </is>
       </c>
       <c r="C6" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="D6" t="n">
+        <v>39</v>
+      </c>
+      <c r="E6" t="n">
+        <v>582</v>
+      </c>
+      <c r="F6" t="n">
         <v>5</v>
       </c>
-      <c r="E6" t="n">
-        <v>130</v>
-      </c>
-      <c r="F6" t="n">
-        <v>2</v>
-      </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>2/3</t>
+          <t>5/6</t>
         </is>
       </c>
       <c r="H6" t="n">
@@ -5520,12 +5544,12 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>ATU Main Campus</t>
+          <t>City Campus</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Racheal Boamah</t>
+          <t>Abednego Abbey</t>
         </is>
       </c>
       <c r="C7" t="n">
@@ -5535,47 +5559,47 @@
         <v>28</v>
       </c>
       <c r="E7" t="n">
-        <v>970</v>
+        <v>465</v>
       </c>
       <c r="F7" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>4/6</t>
+          <t>6/6</t>
         </is>
       </c>
       <c r="H7" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="I7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>City Campus</t>
+          <t>Jamestown</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Abednego Abbey</t>
+          <t>Joel Quartey</t>
         </is>
       </c>
       <c r="C8" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="D8" t="n">
-        <v>22</v>
+        <v>11</v>
       </c>
       <c r="E8" t="n">
-        <v>210</v>
+        <v>70</v>
       </c>
       <c r="F8" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>5/5</t>
+          <t>3/3</t>
         </is>
       </c>
       <c r="H8" t="n">
@@ -5586,29 +5610,29 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Jamestown</t>
+          <t>Jamestown Allos</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Joel Quartey</t>
+          <t>Ishmael Oplerm</t>
         </is>
       </c>
       <c r="C9" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="D9" t="n">
-        <v>10</v>
+        <v>17</v>
       </c>
       <c r="E9" t="n">
-        <v>50</v>
+        <v>350</v>
       </c>
       <c r="F9" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>3/3</t>
+          <t>5/5</t>
         </is>
       </c>
       <c r="H9" t="n">
@@ -5619,29 +5643,29 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Jamestown Allos</t>
+          <t>UssherFort</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Ishmael Oplerm</t>
+          <t>Seth Kpelebe</t>
         </is>
       </c>
       <c r="C10" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="D10" t="n">
-        <v>21</v>
+        <v>10</v>
       </c>
       <c r="E10" t="n">
-        <v>465</v>
+        <v>110</v>
       </c>
       <c r="F10" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>5/5</t>
+          <t>3/3</t>
         </is>
       </c>
       <c r="H10" t="n">
@@ -5652,29 +5676,29 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>UssherFort</t>
+          <t>Yours and Ours</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Seth Kpelebe</t>
+          <t>Prince Odum</t>
         </is>
       </c>
       <c r="C11" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D11" t="n">
         <v>7</v>
       </c>
       <c r="E11" t="n">
-        <v>100</v>
+        <v>230</v>
       </c>
       <c r="F11" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>3/3</t>
+          <t>2/2</t>
         </is>
       </c>
       <c r="H11" t="n">
@@ -5685,64 +5709,31 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Yours and Ours</t>
-        </is>
-      </c>
-      <c r="B12" t="inlineStr">
-        <is>
-          <t>Prince Odum</t>
-        </is>
-      </c>
-      <c r="C12" t="n">
-        <v>2</v>
-      </c>
-      <c r="D12" t="n">
-        <v>8</v>
-      </c>
-      <c r="E12" t="n">
-        <v>60</v>
-      </c>
-      <c r="F12" t="n">
-        <v>2</v>
-      </c>
-      <c r="G12" t="inlineStr">
-        <is>
-          <t>2/2</t>
-        </is>
-      </c>
-      <c r="H12" t="n">
-        <v>0</v>
-      </c>
-      <c r="I12" t="inlineStr"/>
-    </row>
-    <row r="13">
-      <c r="A13" t="inlineStr">
-        <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="C13">
-        <f>SUM(C3:C12)</f>
-        <v/>
-      </c>
-      <c r="D13">
-        <f>SUM(D3:D12)</f>
-        <v/>
-      </c>
-      <c r="E13">
-        <f>SUM(E3:E12)</f>
-        <v/>
-      </c>
-      <c r="F13">
-        <f>SUM(F3:F12)</f>
-        <v/>
-      </c>
-      <c r="G13">
-        <f>F13&amp;"/"&amp;C13</f>
-        <v/>
-      </c>
-      <c r="H13">
-        <f>SUM(H3:H12)</f>
+      <c r="C12">
+        <f>SUM(C3:C11)</f>
+        <v/>
+      </c>
+      <c r="D12">
+        <f>SUM(D3:D11)</f>
+        <v/>
+      </c>
+      <c r="E12">
+        <f>SUM(E3:E11)</f>
+        <v/>
+      </c>
+      <c r="F12">
+        <f>SUM(F3:F11)</f>
+        <v/>
+      </c>
+      <c r="G12">
+        <f>F12&amp;"/"&amp;C12</f>
+        <v/>
+      </c>
+      <c r="H12">
+        <f>SUM(H3:H11)</f>
         <v/>
       </c>
     </row>
@@ -5829,21 +5820,21 @@
         <v>1</v>
       </c>
       <c r="D3" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="E3" t="n">
-        <v>13</v>
+        <v>0</v>
       </c>
       <c r="F3" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>1/1</t>
+          <t>0/1</t>
         </is>
       </c>
       <c r="H3" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I3" t="inlineStr"/>
     </row>
@@ -5862,21 +5853,21 @@
         <v>3</v>
       </c>
       <c r="D4" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="E4" t="n">
-        <v>30</v>
+        <v>15</v>
       </c>
       <c r="F4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>3/3</t>
+          <t>2/3</t>
         </is>
       </c>
       <c r="H4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I4" t="inlineStr"/>
     </row>
@@ -5895,10 +5886,10 @@
         <v>2</v>
       </c>
       <c r="D5" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="E5" t="n">
-        <v>45</v>
+        <v>70</v>
       </c>
       <c r="F5" t="n">
         <v>2</v>
@@ -5928,10 +5919,10 @@
         <v>3</v>
       </c>
       <c r="D6" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="E6" t="n">
-        <v>195</v>
+        <v>40</v>
       </c>
       <c r="F6" t="n">
         <v>3</v>
@@ -5997,18 +5988,18 @@
         <v>11</v>
       </c>
       <c r="E8" t="n">
-        <v>70</v>
+        <v>60</v>
       </c>
       <c r="F8" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>2/4</t>
+          <t>3/4</t>
         </is>
       </c>
       <c r="H8" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="I8" t="inlineStr"/>
     </row>
@@ -6027,21 +6018,21 @@
         <v>3</v>
       </c>
       <c r="D9" t="n">
-        <v>17</v>
+        <v>13</v>
       </c>
       <c r="E9" t="n">
-        <v>140</v>
+        <v>110</v>
       </c>
       <c r="F9" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>3/3</t>
+          <t>2/3</t>
         </is>
       </c>
       <c r="H9" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I9" t="inlineStr"/>
     </row>
@@ -6060,10 +6051,10 @@
         <v>2</v>
       </c>
       <c r="D10" t="n">
-        <v>10</v>
+        <v>7</v>
       </c>
       <c r="E10" t="n">
-        <v>60</v>
+        <v>55</v>
       </c>
       <c r="F10" t="n">
         <v>2</v>
@@ -6096,7 +6087,7 @@
         <v>9</v>
       </c>
       <c r="E11" t="n">
-        <v>25</v>
+        <v>31</v>
       </c>
       <c r="F11" t="n">
         <v>2</v>
@@ -6126,21 +6117,21 @@
         <v>7</v>
       </c>
       <c r="D12" t="n">
-        <v>12</v>
+        <v>2</v>
       </c>
       <c r="E12" t="n">
-        <v>45</v>
+        <v>10</v>
       </c>
       <c r="F12" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>3/7</t>
+          <t>1/7</t>
         </is>
       </c>
       <c r="H12" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="I12" t="inlineStr"/>
     </row>
@@ -6159,21 +6150,21 @@
         <v>6</v>
       </c>
       <c r="D13" t="n">
-        <v>22</v>
+        <v>0</v>
       </c>
       <c r="E13" t="n">
-        <v>611</v>
+        <v>0</v>
       </c>
       <c r="F13" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>5/6</t>
+          <t>0/6</t>
         </is>
       </c>
       <c r="H13" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="I13" t="inlineStr"/>
     </row>
@@ -6192,21 +6183,21 @@
         <v>2</v>
       </c>
       <c r="D14" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="E14" t="n">
-        <v>70</v>
+        <v>80</v>
       </c>
       <c r="F14" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>1/2</t>
+          <t>2/2</t>
         </is>
       </c>
       <c r="H14" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I14" t="inlineStr"/>
     </row>
@@ -6225,21 +6216,21 @@
         <v>4</v>
       </c>
       <c r="D15" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="E15" t="n">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="F15" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>1/4</t>
+          <t>0/4</t>
         </is>
       </c>
       <c r="H15" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="I15" t="inlineStr"/>
     </row>

</xml_diff>